<commit_message>
pre day in life pivot
</commit_message>
<xml_diff>
--- a/ProxyMap/Api routing.xlsx
+++ b/ProxyMap/Api routing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JeremyJoyner\code\deptorientation\ProxyMap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8611C714-7F8F-4585-914A-87669343E5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7ACEC7-88BF-4A6F-AA9F-CFA3D8D12A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2745" yWindow="1500" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{E193D418-9444-4EFB-87E3-D74577144D85}"/>
   </bookViews>
@@ -147,12 +147,40 @@
     <t>Selector save (per tracker row)</t>
   </si>
   <si>
+    <r>
+      <t>/api/orientation-tracker/item/[itemId]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (POST)</t>
+    </r>
+  </si>
+  <si>
     <t>(Tracker Item Update function)</t>
   </si>
   <si>
     <t>“Mark Orientation as Reviewed”</t>
   </si>
   <si>
+    <r>
+      <t>/api/employees/reviewed/[id]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (POST)</t>
+    </r>
+  </si>
+  <si>
     <t>EmployeeProfileReviewed</t>
   </si>
   <si>
@@ -332,9 +360,6 @@
   </si>
   <si>
     <t>Screen / Action</t>
-  </si>
-  <si>
-    <t>Next API Route</t>
   </si>
   <si>
     <r>
@@ -361,37 +386,34 @@
     </r>
   </si>
   <si>
-    <t>Returns id, name, roleCode, reviewed, reviewAudit, modified</t>
-  </si>
-  <si>
     <t>Create New Employee</t>
   </si>
   <si>
-    <t>/api/employees</t>
-  </si>
-  <si>
-    <t>Creates EmployeeProfiles item</t>
-  </si>
-  <si>
     <t>Release Orientation Items</t>
   </si>
   <si>
-    <t>/api/orientation-tracker/release/[id]</t>
-  </si>
-  <si>
     <t>OrientationUpdater</t>
   </si>
   <si>
-    <t>Generates OrientationTracker items</t>
-  </si>
-  <si>
     <t>Employee Detail Header</t>
   </si>
   <si>
     <t>/api/employees/[id]</t>
   </si>
   <si>
-    <t>EmployeeProfilesGet</t>
+    <t>/api/orientation-tracker/[id]</t>
+  </si>
+  <si>
+    <t>OrientationTrackerItemUpdate</t>
+  </si>
+  <si>
+    <t>/api/audit/reviewed</t>
+  </si>
+  <si>
+    <t>Next.js API Route</t>
+  </si>
+  <si>
+    <t>Purpose / Data Flow</t>
   </si>
   <si>
     <r>
@@ -403,6 +425,62 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
+      <t>{ id, name, roleCode, reviewed, reviewAudit, modified }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>. Powers full employees table.</t>
+    </r>
+  </si>
+  <si>
+    <t>Creates EmployeeProfiles item (Title, RoleLookupId, StartDate, SupervisorLookupId).</t>
+  </si>
+  <si>
+    <r>
+      <t>/api/orientation-tracker/release/[id]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (POST)</t>
+    </r>
+  </si>
+  <si>
+    <t>Generates OrientationTracker checklist items for an employee based on Role template.</t>
+  </si>
+  <si>
+    <r>
+      <t>EmployeeProfilesGet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (plural version)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Returns one employee with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
       <t>{ id, fields }</t>
     </r>
     <r>
@@ -412,50 +490,90 @@
         <rFont val="Segoe UI"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> for one employee</t>
-    </r>
-  </si>
-  <si>
-    <t>Orientation Items (per employee)</t>
-  </si>
-  <si>
-    <t>/api/orientation-tracker/[id]</t>
-  </si>
-  <si>
-    <t>Loads tracker rows</t>
-  </si>
-  <si>
-    <t>Update Tracker Item</t>
-  </si>
-  <si>
-    <t>/api/orientation-tracker/item/[itemId]</t>
-  </si>
-  <si>
-    <t>OrientationTrackerItemUpdate</t>
-  </si>
-  <si>
-    <t>Updates Status</t>
-  </si>
-  <si>
-    <t>Supervisor Clicks “Mark Orientation as Reviewed”</t>
-  </si>
-  <si>
-    <t>/api/audit/reviewed</t>
-  </si>
-  <si>
-    <t>NONE (local no‑op)</t>
-  </si>
-  <si>
-    <t>Logs audit event (now fixed)</t>
-  </si>
-  <si>
-    <t>Then →</t>
-  </si>
-  <si>
-    <t>/api/employees/reviewed/[id]</t>
-  </si>
-  <si>
-    <t>Writes Reviewed="Yes", ReviewAudit timestamp</t>
+      <t xml:space="preserve"> for detail header.</t>
+    </r>
+  </si>
+  <si>
+    <t>Orientation Items (General + Dept)</t>
+  </si>
+  <si>
+    <t>Returns checklist rows (Status, TemplateTaskId, Category, etc.) used to render the 3‑state selector.</t>
+  </si>
+  <si>
+    <t>Update Single Tracker Item</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PATCHes </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> field on a single OrientationTracker list item. Retry with snake_case if needed.</t>
+    </r>
+  </si>
+  <si>
+    <t>Audit Log (pre‑review)</t>
+  </si>
+  <si>
+    <t>NONE — local no‑op</t>
+  </si>
+  <si>
+    <t>UI requires this call. Logs locally for now (successful 200). Can later become real audit logging function.</t>
+  </si>
+  <si>
+    <t>Mark Orientation as Reviewed</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PATCHes EmployeeProfiles → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Reviewed = true/false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ReviewAudit = ISO timestamp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>. Supports boolean &amp; fallback string values for compatibility with Yes/No or Choice columns.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -947,26 +1065,26 @@
         <v>6</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="29.25" thickBot="1">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29.25" thickBot="1">
       <c r="A4" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>18</v>
@@ -983,27 +1101,27 @@
         <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="29.25" thickBot="1">
       <c r="A6" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1019,26 +1137,26 @@
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
     <col min="2" max="2" width="38.85546875" customWidth="1"/>
     <col min="3" max="3" width="39.7109375" customWidth="1"/>
-    <col min="4" max="4" width="62.140625" customWidth="1"/>
+    <col min="4" max="4" width="78.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
@@ -1047,7 +1165,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
@@ -1055,94 +1173,94 @@
         <v>38</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A4" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A6" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A7" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
       <c r="A8" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="32.25" customHeight="1" thickBot="1">
-      <c r="A9" s="3" t="s">
-        <v>60</v>
+      <c r="A9" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>62</v>

</xml_diff>